<commit_message>
fix all pipeline l1 - 0909
</commit_message>
<xml_diff>
--- a/project/data/entities/entities.xlsx
+++ b/project/data/entities/entities.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30431"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30502"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fptscomvn.sharepoint.com/sites/FRA_DataIngestion/Shared Documents/AnPT/news-scape/project/data/entities/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="11_EA5ECF2F241B686E4F08FDD2D22E83478481117C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B65BF4DB-CE59-4BB2-ACF3-331D6AF05C8F}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="11_EA5ECF2F241B686E4F08FDD2D22E83478481117C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DCA6DF09-F211-4B42-A543-C96DAA213533}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="5" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="_Huong_dan" sheetId="1" r:id="rId1"/>
@@ -81091,12 +81091,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="540cf7b3-6f7a-4cd3-95f1-edd8c1c86d9a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c36903d5-5ed0-4454-a196-b1a2f9ebaa03">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -81281,18 +81283,16 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="540cf7b3-6f7a-4cd3-95f1-edd8c1c86d9a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c36903d5-5ed0-4454-a196-b1a2f9ebaa03">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5378DDAD-865F-42DE-A82B-00E9C0DD2B8F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F84C9C32-2D24-4AF2-BC49-7B28A25B8B7F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -81300,5 +81300,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F84C9C32-2D24-4AF2-BC49-7B28A25B8B7F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5378DDAD-865F-42DE-A82B-00E9C0DD2B8F}"/>
 </file>
</xml_diff>